<commit_message>
feat: support list and singleton Luban tables
</commit_message>
<xml_diff>
--- a/config/luban/Datas/__tables__.xlsx
+++ b/config/luban/Datas/__tables__.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="20.375" customWidth="1" style="2" min="2" max="2"/>
@@ -572,6 +572,78 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>game.TbRotationMessage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RotationMessage</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>#game.rotation_message.xlsx</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>list</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>轮播消息列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>game.TbGameGlobal</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GameGlobal</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>#game.game_global.xlsx</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>one</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>全局单例配置</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>